<commit_message>
Guardo el estado de main.py con el que corri las pruebas del tercer experimento para poder ver si hay o no un problema en el analisis que hace que las predicciones sean tan altas.
</commit_message>
<xml_diff>
--- a/modeling/data/inglaterra/df_modelos.xlsx
+++ b/modeling/data/inglaterra/df_modelos.xlsx
@@ -455,10 +455,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>41.31578947368421</v>
+        <v>70.55383556931545</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.8394736842104908</v>
+        <v>79.21740689121256</v>
       </c>
     </row>
     <row r="3">
@@ -471,10 +471,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>50.17543859649123</v>
+        <v>75.79979360165119</v>
       </c>
       <c r="D3" t="n">
-        <v>-1.516666666666644</v>
+        <v>85.11832132741512</v>
       </c>
     </row>
     <row r="4">
@@ -497,10 +497,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>48.7719298245614</v>
+        <v>78.24217406260749</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3956140350877185</v>
+        <v>97.97347249615856</v>
       </c>
     </row>
     <row r="5">
@@ -513,10 +513,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>52.45614035087719</v>
+        <v>54.04196766425869</v>
       </c>
       <c r="D5" t="n">
-        <v>-5.047368421052594</v>
+        <v>9.325228326396866</v>
       </c>
     </row>
     <row r="6">
@@ -529,10 +529,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>50.35087719298246</v>
+        <v>54.19676642586859</v>
       </c>
       <c r="D6" t="n">
-        <v>-9.509649122807005</v>
+        <v>11.11522829837297</v>
       </c>
     </row>
     <row r="7">
@@ -546,10 +546,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50.26315789473684</v>
+        <v>54.04196766425869</v>
       </c>
       <c r="D7" t="n">
-        <v>-3.109649122806991</v>
+        <v>9.325228326396866</v>
       </c>
     </row>
     <row r="8">
@@ -562,10 +562,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>49.12280701754386</v>
+        <v>79.82456140350878</v>
       </c>
       <c r="D8" t="n">
-        <v>4.165789473684221</v>
+        <v>103.2173665450061</v>
       </c>
     </row>
   </sheetData>

</xml_diff>